<commit_message>
The record is the clean run: every output regenerated from the committed code on a clean checkout, with its report
The committed calibration had been produced before the sigma floor entered
adopted_model.scale_block, so the committed code did not reproduce the committed
results: a full-manifest run from a fresh clone of 1387124 (57 scripts, no failures,
4.6 hours) moved the posterior summaries at the third decimal (k 0.615 to 0.614,
gamma 0.244 to 0.240) and every downstream figure with them. Those outputs, and the
run report that records them, replace the earlier ones; a second calibration run from
the same code reproduces the posterior draws byte for byte. The data-audit document
is regenerated from the new exposure file.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vignettes/vignette-1/decomposition_summary.xlsx
+++ b/vignettes/vignette-1/decomposition_summary.xlsx
@@ -458,16 +458,16 @@
         <v>0.07244399999999999</v>
       </c>
       <c r="C2" t="n">
-        <v>0.06721199999999999</v>
+        <v>0.067217</v>
       </c>
       <c r="D2" t="n">
-        <v>0.064022</v>
+        <v>0.06408800000000001</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.004278</v>
+        <v>-0.004262</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.004144</v>
+        <v>-0.004094</v>
       </c>
     </row>
     <row r="3">
@@ -480,16 +480,16 @@
         <v>0.766024</v>
       </c>
       <c r="C3" t="n">
-        <v>0.409409</v>
+        <v>0.408942</v>
       </c>
       <c r="D3" t="n">
-        <v>0.385686</v>
+        <v>0.38559</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.331654</v>
+        <v>-0.332446</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.048684</v>
+        <v>-0.047988</v>
       </c>
     </row>
     <row r="4">
@@ -502,16 +502,16 @@
         <v>0.865683</v>
       </c>
       <c r="C4" t="n">
-        <v>0.646715</v>
+        <v>0.646491</v>
       </c>
       <c r="D4" t="n">
-        <v>0.600541</v>
+        <v>0.601285</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.193477</v>
+        <v>-0.19389</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.07166500000000001</v>
+        <v>-0.070508</v>
       </c>
     </row>
   </sheetData>

</xml_diff>